<commit_message>
Update all processed Excel files to 48-company portfolio
</commit_message>
<xml_diff>
--- a/data/processed/Financial Exposure.xlsx
+++ b/data/processed/Financial Exposure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bocconi.sharepoint.com/sites/Geopolitics-DataGroup1/Documenti condivisi/General/Final Dataset - CGPR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C91DB5-5FA0-1644-B9FC-DA994EA1695C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{66C91DB5-5FA0-1644-B9FC-DA994EA1695C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AF77051-6C0A-4B46-880F-56E448D1EC2D}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Financial Exposure" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>Company</t>
   </si>
@@ -120,6 +120,75 @@
   </si>
   <si>
     <t>Volkswagen</t>
+  </si>
+  <si>
+    <t>Leonardo</t>
+  </si>
+  <si>
+    <t>Pfizer</t>
+  </si>
+  <si>
+    <t>Prysmian</t>
+  </si>
+  <si>
+    <t>Unicredit</t>
+  </si>
+  <si>
+    <t>Campari</t>
+  </si>
+  <si>
+    <t>Moncler</t>
+  </si>
+  <si>
+    <t>Ferrari</t>
+  </si>
+  <si>
+    <t>Alibaba</t>
+  </si>
+  <si>
+    <t>Nestlè</t>
+  </si>
+  <si>
+    <t>Gazprom</t>
+  </si>
+  <si>
+    <t>Novartis</t>
+  </si>
+  <si>
+    <t>Moderna</t>
+  </si>
+  <si>
+    <t>HSBC</t>
+  </si>
+  <si>
+    <t>Walmart</t>
+  </si>
+  <si>
+    <t>Unilever</t>
+  </si>
+  <si>
+    <t>Coca-Cola</t>
+  </si>
+  <si>
+    <t>Caterpillar</t>
+  </si>
+  <si>
+    <t>Tesla</t>
+  </si>
+  <si>
+    <t>Alphabet</t>
+  </si>
+  <si>
+    <t>Saudi Aramco</t>
+  </si>
+  <si>
+    <t>Shell</t>
+  </si>
+  <si>
+    <t>Chevron</t>
+  </si>
+  <si>
+    <t>ExxonMobil</t>
   </si>
 </sst>
 </file>
@@ -140,15 +209,21 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -171,14 +246,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -196,8 +292,8 @@
         <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -224,6 +320,7 @@
         <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
@@ -311,15 +408,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{972B53DE-EEB5-614E-80EB-EE4E321B6086}" name="Tabella1" displayName="Tabella1" ref="A1:C26" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="A1:C26" xr:uid="{972B53DE-EEB5-614E-80EB-EE4E321B6086}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{972B53DE-EEB5-614E-80EB-EE4E321B6086}" name="Tabella1" displayName="Tabella1" ref="A1:C49" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="A1:C49" xr:uid="{972B53DE-EEB5-614E-80EB-EE4E321B6086}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B26">
     <sortCondition ref="A1:A26"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{A737B249-4BB7-3843-8591-B8CBE2EE111B}" name="Company" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{85548CF2-8672-E24C-998E-BFAE291A91B1}" name="Net Debt/EBITDA 2024" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{B9B40A37-3F4D-1446-92C3-D5C502D24C60}" name="Financial Exposure - Multiplier" dataDxfId="0">
+    <tableColumn id="2" xr3:uid="{85548CF2-8672-E24C-998E-BFAE291A91B1}" name="Net Debt/EBITDA 2024" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{B9B40A37-3F4D-1446-92C3-D5C502D24C60}" name="Financial Exposure - Multiplier" dataDxfId="1">
       <calculatedColumnFormula xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -612,7 +709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="18" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -635,7 +732,7 @@
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="6">
         <v>1.45</v>
       </c>
       <c r="C2" s="2">
@@ -647,7 +744,7 @@
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="6">
         <v>0.35</v>
       </c>
       <c r="C3" s="2">
@@ -659,7 +756,7 @@
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="6">
         <v>-0.35</v>
       </c>
       <c r="C4" s="2">
@@ -671,7 +768,7 @@
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="6">
         <v>-0.72</v>
       </c>
       <c r="C5" s="2">
@@ -683,7 +780,7 @@
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="6">
         <v>5.0999999999999996</v>
       </c>
       <c r="C6" s="2">
@@ -695,7 +792,7 @@
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="6">
         <v>2.15</v>
       </c>
       <c r="C7" s="2">
@@ -707,7 +804,7 @@
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="6">
         <v>1.69</v>
       </c>
       <c r="C8" s="2">
@@ -719,7 +816,7 @@
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="6">
         <v>-0.57999999999999996</v>
       </c>
       <c r="C9" s="2">
@@ -731,7 +828,7 @@
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="6">
         <v>-0.56999999999999995</v>
       </c>
       <c r="C10" s="2">
@@ -743,7 +840,7 @@
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="6">
         <v>0.44</v>
       </c>
       <c r="C11" s="2">
@@ -755,7 +852,7 @@
       <c r="A12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="6">
         <v>1.02</v>
       </c>
       <c r="C12" s="2">
@@ -767,7 +864,7 @@
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="6">
         <v>-0.32</v>
       </c>
       <c r="C13" s="2">
@@ -779,7 +876,7 @@
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="6">
         <v>0.16</v>
       </c>
       <c r="C14" s="2">
@@ -791,7 +888,7 @@
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="6">
         <v>0.52</v>
       </c>
       <c r="C15" s="2">
@@ -803,7 +900,7 @@
       <c r="A16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="6">
         <v>-0.39</v>
       </c>
       <c r="C16" s="2">
@@ -815,7 +912,7 @@
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="6">
         <v>1.1000000000000001</v>
       </c>
       <c r="C17" s="2">
@@ -827,7 +924,7 @@
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="6">
         <v>0.87</v>
       </c>
       <c r="C18" s="2">
@@ -839,7 +936,7 @@
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="6">
         <v>-1.24</v>
       </c>
       <c r="C19" s="2">
@@ -851,7 +948,7 @@
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="6">
         <v>-0.02</v>
       </c>
       <c r="C20" s="2">
@@ -863,7 +960,7 @@
       <c r="A21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="6">
         <v>0.76</v>
       </c>
       <c r="C21" s="2">
@@ -875,7 +972,7 @@
       <c r="A22" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="6">
         <v>0.06</v>
       </c>
       <c r="C22" s="2">
@@ -887,7 +984,7 @@
       <c r="A23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="6">
         <v>0.44</v>
       </c>
       <c r="C23" s="2">
@@ -899,7 +996,7 @@
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="6">
         <v>-1.17</v>
       </c>
       <c r="C24" s="2">
@@ -911,7 +1008,7 @@
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="6">
         <v>-0.69</v>
       </c>
       <c r="C25" s="2">
@@ -923,7 +1020,7 @@
       <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="6">
         <v>-1</v>
       </c>
       <c r="C26" s="2">
@@ -931,8 +1028,284 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="7">
+        <v>0.9</v>
+      </c>
+      <c r="C27" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="7">
+        <v>1.6</v>
+      </c>
+      <c r="C28" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C29" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="7">
+        <v>3.5</v>
+      </c>
+      <c r="C30" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="C31" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="7">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="C33" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="7">
+        <v>1</v>
+      </c>
+      <c r="C34" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C35" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="C36" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="7">
+        <v>1.3</v>
+      </c>
+      <c r="C37" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="C38" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="7">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="C39" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" s="7">
+        <v>1.5</v>
+      </c>
+      <c r="C40" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="7">
+        <v>2.5</v>
+      </c>
+      <c r="C41" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A42" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="7">
+        <v>2.4</v>
+      </c>
+      <c r="C42" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B43" s="7">
+        <v>1.8</v>
+      </c>
+      <c r="C43" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A44" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B44" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="C44" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="7">
+        <v>1.8</v>
+      </c>
+      <c r="C45" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A46" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="C46" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B47" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="C47" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A48" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B48" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="C48" s="3">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="19" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B49" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="C49" s="5">
+        <f xml:space="preserve"> IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;0, 0.8,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;2, 0.9, IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]] &lt; 4, 1,IF(Tabella1[[#This Row],[Net Debt/EBITDA 2024]]&lt;6,1.1,1.2))))</f>
+        <v>0.9</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C26">
+  <conditionalFormatting sqref="C2:C49">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -952,6 +1325,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100086DC0FFDEFA864DA147FFDEA823F2EE" ma:contentTypeVersion="3" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="efa000e167d9ce5db8cd2eb5b6f87cd4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f94584ddf2c7798ba84aeef6e679263" ns2:_="">
     <xsd:import namespace="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39"/>
@@ -1089,22 +1477,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FE50425-CE3F-4044-94E1-4363C82699D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A65F6982-0AB8-4F18-B8A2-A0502C83FF9D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F14E50ED-5E40-4117-8E72-7B12F1FBEEDA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1120,28 +1517,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A65F6982-0AB8-4F18-B8A2-A0502C83FF9D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FE50425-CE3F-4044-94E1-4363C82699D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>